<commit_message>
Update 2024-09-20018D Source Data Ext. Fig. 7.xlsx
1
</commit_message>
<xml_diff>
--- a/2024-09-20018D Source Data Ext. Fig. 7.xlsx
+++ b/2024-09-20018D Source Data Ext. Fig. 7.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ytian\Desktop\To be revised\Source data\Clean version\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Source Data_Proof\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14B97842-5A25-4C60-AAD4-522A5B154FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14EACD7B-6053-488B-A479-0CDF4C977625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1063,10 +1063,10 @@
         <v>0.83</v>
       </c>
       <c r="U3" s="10">
-        <v>5.9</v>
+        <v>5.87</v>
       </c>
       <c r="V3" s="10">
-        <v>6.9</v>
+        <v>6.94</v>
       </c>
       <c r="W3" s="10">
         <v>13</v>
@@ -1193,13 +1193,13 @@
         <v>0.71</v>
       </c>
       <c r="U5" s="10">
-        <v>5.9</v>
+        <v>5.94</v>
       </c>
       <c r="V5" s="10">
-        <v>5.9</v>
+        <v>5.88</v>
       </c>
       <c r="W5" s="10">
-        <v>7.1</v>
+        <v>7.09</v>
       </c>
     </row>
     <row r="6" spans="1:23">

</xml_diff>